<commit_message>
Eindcontrole scrapers matchmaking enrich upload template en tests opgeschoond
</commit_message>
<xml_diff>
--- a/public/templates/fightsupport-upload.xlsx
+++ b/public/templates/fightsupport-upload.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vecht\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Apps\Fightsupport\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B40675-3BD3-4635-8177-0F74513820C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A65DFB-712C-43AA-84BF-C79A02DC560D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{729028DD-135B-4EB2-BD2B-100D9B9B9271}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{729028DD-135B-4EB2-BD2B-100D9B9B9271}"/>
   </bookViews>
   <sheets>
     <sheet name="Upload" sheetId="1" r:id="rId1"/>
@@ -30,12 +30,15 @@
         <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="72">
   <si>
     <t xml:space="preserve">FIGHTSUPPORT UPLOAD EXCEL </t>
   </si>
@@ -255,6 +258,15 @@
   </si>
   <si>
     <t xml:space="preserve">Vergeet niet om een 0 in partij nummer te zetten. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sportscholen buiten nederlands: </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zet achter de sportschool tussen haakjes de land afkorting dus achter een Duitse sportschool zet je (DE) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgische sportscholen (BE) of welk land dan ook </t>
   </si>
 </sst>
 </file>
@@ -870,30 +882,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{848D0188-C820-4E97-A405-5753A30365E6}">
   <dimension ref="A1:Q45"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="8.44140625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="11.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.88671875" style="1"/>
-    <col min="8" max="8" width="3.109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.6640625" customWidth="1"/>
-    <col min="10" max="10" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="8.88671875" style="1"/>
-    <col min="17" max="17" width="8.88671875" style="1" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="8.453125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="11.08984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.90625" style="1"/>
+    <col min="8" max="8" width="3.08984375" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.6328125" customWidth="1"/>
+    <col min="10" max="10" width="24.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.453125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="8.90625" style="1"/>
+    <col min="17" max="17" width="8.90625" style="1" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" ht="18.5" x14ac:dyDescent="0.45">
       <c r="D1" s="18"/>
       <c r="E1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" ht="16" x14ac:dyDescent="0.4">
       <c r="E2" s="4" t="s">
         <v>1</v>
       </c>
@@ -905,7 +917,7 @@
       <c r="K2" s="6"/>
       <c r="L2" s="9"/>
     </row>
-    <row r="3" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" ht="16" x14ac:dyDescent="0.4">
       <c r="E3" s="4" t="s">
         <v>3</v>
       </c>
@@ -917,7 +929,7 @@
       <c r="K3" s="6"/>
       <c r="L3" s="9"/>
     </row>
-    <row r="4" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" ht="16" x14ac:dyDescent="0.35">
       <c r="E4" s="16" t="s">
         <v>5</v>
       </c>
@@ -929,10 +941,10 @@
       <c r="K4" s="6"/>
       <c r="L4" s="9"/>
     </row>
-    <row r="5" spans="1:17" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" ht="16" x14ac:dyDescent="0.35">
       <c r="K5" s="7"/>
     </row>
-    <row r="6" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
@@ -976,7 +988,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H7" s="3" t="s">
         <v>20</v>
       </c>
@@ -984,7 +996,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H8" s="3" t="s">
         <v>20</v>
       </c>
@@ -992,7 +1004,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H9" s="3" t="s">
         <v>20</v>
       </c>
@@ -1000,7 +1012,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H10" s="3" t="s">
         <v>20</v>
       </c>
@@ -1008,7 +1020,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H11" s="3" t="s">
         <v>20</v>
       </c>
@@ -1016,7 +1028,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1024,7 +1036,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H13" s="3" t="s">
         <v>20</v>
       </c>
@@ -1032,7 +1044,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H14" s="3" t="s">
         <v>20</v>
       </c>
@@ -1040,7 +1052,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H15" s="3" t="s">
         <v>20</v>
       </c>
@@ -1048,7 +1060,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
       <c r="H16" s="3" t="s">
         <v>20</v>
       </c>
@@ -1056,7 +1068,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H17" s="3" t="s">
         <v>20</v>
       </c>
@@ -1064,7 +1076,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="18" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H18" s="3" t="s">
         <v>20</v>
       </c>
@@ -1072,7 +1084,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="19" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="19" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H19" s="3" t="s">
         <v>20</v>
       </c>
@@ -1080,7 +1092,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="20" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H20" s="3" t="s">
         <v>20</v>
       </c>
@@ -1088,7 +1100,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="21" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="21" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H21" s="3" t="s">
         <v>20</v>
       </c>
@@ -1096,7 +1108,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="22" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="22" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H22" s="3" t="s">
         <v>20</v>
       </c>
@@ -1104,7 +1116,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="23" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="23" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H23" s="3" t="s">
         <v>20</v>
       </c>
@@ -1112,7 +1124,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="24" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="24" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H24" s="3" t="s">
         <v>20</v>
       </c>
@@ -1120,7 +1132,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="25" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="25" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1128,7 +1140,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="26" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="26" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H26" s="3" t="s">
         <v>20</v>
       </c>
@@ -1136,7 +1148,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="27" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="27" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H27" s="3" t="s">
         <v>20</v>
       </c>
@@ -1144,7 +1156,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="28" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H28" s="3" t="s">
         <v>20</v>
       </c>
@@ -1152,7 +1164,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="29" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H29" s="3" t="s">
         <v>20</v>
       </c>
@@ -1160,7 +1172,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="30" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="30" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H30" s="3" t="s">
         <v>20</v>
       </c>
@@ -1168,7 +1180,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="31" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="31" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H31" s="3" t="s">
         <v>20</v>
       </c>
@@ -1176,7 +1188,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="32" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="32" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H32" s="3" t="s">
         <v>20</v>
       </c>
@@ -1184,7 +1196,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="33" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="33" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H33" s="3" t="s">
         <v>20</v>
       </c>
@@ -1192,7 +1204,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="34" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="34" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H34" s="3" t="s">
         <v>20</v>
       </c>
@@ -1200,7 +1212,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="35" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="35" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H35" s="3" t="s">
         <v>20</v>
       </c>
@@ -1208,7 +1220,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="36" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="36" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H36" s="3" t="s">
         <v>20</v>
       </c>
@@ -1216,7 +1228,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="37" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="37" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H37" s="3" t="s">
         <v>20</v>
       </c>
@@ -1224,7 +1236,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="38" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H38" s="3" t="s">
         <v>20</v>
       </c>
@@ -1232,7 +1244,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="39" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="39" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H39" s="3" t="s">
         <v>20</v>
       </c>
@@ -1240,7 +1252,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="40" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H40" s="3" t="s">
         <v>20</v>
       </c>
@@ -1248,7 +1260,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="41" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="41" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H41" s="3" t="s">
         <v>20</v>
       </c>
@@ -1256,22 +1268,22 @@
         <v>62</v>
       </c>
     </row>
-    <row r="42" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="42" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H42" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="43" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="43" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H43" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="44" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="44" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H44" s="3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="45" spans="8:17" x14ac:dyDescent="0.3">
+    <row r="45" spans="8:17" x14ac:dyDescent="0.35">
       <c r="H45" s="3" t="s">
         <v>20</v>
       </c>
@@ -1291,10 +1303,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{37F0FFA5-DB3B-44A4-9CBE-730EE37B6DAC}">
-  <dimension ref="A1:L28"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L33"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:12" ht="18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A1" s="17" t="s">
         <v>21</v>
       </c>
@@ -1302,32 +1314,32 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -1335,24 +1347,39 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" ht="16" x14ac:dyDescent="0.4">
       <c r="A28" s="2" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="16" x14ac:dyDescent="0.4">
+      <c r="A31" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>